<commit_message>
Results from the changes/lessons
</commit_message>
<xml_diff>
--- a/data/01_metadata_INERA_stations/metadata_INERA_stations.xlsx
+++ b/data/01_metadata_INERA_stations/metadata_INERA_stations.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://vub-my.sharepoint.com/personal/derrick_muheki_vub_be/Documents/PhD_Derrick_Muheki/21_Research/21_6_Analysis/21_6_0_Preprocessing_data/Data_Rescue_Congo_DRC-1/data/01_metadata_INERA_stations/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="8_{1B0374CF-1AF6-4015-9A17-346A27468979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1E6E4007-AFBF-402B-8F6D-C5213B544D3D}"/>
+  <xr:revisionPtr revIDLastSave="29" documentId="8_{1B0374CF-1AF6-4015-9A17-346A27468979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DF997350-B16B-417C-B2CC-E995947D6127}"/>
   <bookViews>
-    <workbookView xWindow="8064" yWindow="1116" windowWidth="9288" windowHeight="11124" xr2:uid="{0764B754-95B7-4E5B-9740-BD1E6EBCF996}"/>
+    <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8928" xr2:uid="{0764B754-95B7-4E5B-9740-BD1E6EBCF996}"/>
   </bookViews>
   <sheets>
     <sheet name="Stations" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
results of updates to the modules to include precipitation and dry and wet bulb temperatures
</commit_message>
<xml_diff>
--- a/data/01_metadata_INERA_stations/metadata_INERA_stations.xlsx
+++ b/data/01_metadata_INERA_stations/metadata_INERA_stations.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://vub-my.sharepoint.com/personal/derrick_muheki_vub_be/Documents/PhD_Derrick_Muheki/21_Research/21_6_Analysis/21_6_0_Preprocessing_data/Data_Rescue_Congo_DRC-1/data/01_metadata_INERA_stations/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="29" documentId="8_{1B0374CF-1AF6-4015-9A17-346A27468979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DF997350-B16B-417C-B2CC-E995947D6127}"/>
+  <xr:revisionPtr revIDLastSave="30" documentId="8_{1B0374CF-1AF6-4015-9A17-346A27468979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{90C2CE85-9026-4F8F-8E08-677059324097}"/>
   <bookViews>
-    <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8928" xr2:uid="{0764B754-95B7-4E5B-9740-BD1E6EBCF996}"/>
+    <workbookView xWindow="2010" yWindow="1965" windowWidth="24105" windowHeight="18870" xr2:uid="{0764B754-95B7-4E5B-9740-BD1E6EBCF996}"/>
   </bookViews>
   <sheets>
     <sheet name="Stations" sheetId="1" r:id="rId1"/>
@@ -866,7 +866,7 @@
     <t>E 29°47'</t>
   </si>
   <si>
-    <t>Station ID</t>
+    <t>ID</t>
   </si>
 </sst>
 </file>
@@ -1246,18 +1246,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B665FB0-7E50-4F8D-A596-D5F1ADE63703}">
   <dimension ref="A1:H72"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.6640625" customWidth="1"/>
-    <col min="3" max="3" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.7109375" customWidth="1"/>
+    <col min="3" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="19" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1283,7 +1283,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -1309,7 +1309,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -1335,7 +1335,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -1361,7 +1361,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -1387,7 +1387,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>22</v>
       </c>
@@ -1413,7 +1413,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>25</v>
       </c>
@@ -1439,7 +1439,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>214</v>
       </c>
@@ -1465,7 +1465,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>32</v>
       </c>
@@ -1491,7 +1491,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>34</v>
       </c>
@@ -1517,7 +1517,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>215</v>
       </c>
@@ -1543,7 +1543,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>216</v>
       </c>
@@ -1569,7 +1569,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>217</v>
       </c>
@@ -1595,7 +1595,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>41</v>
       </c>
@@ -1621,7 +1621,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>43</v>
       </c>
@@ -1647,7 +1647,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>45</v>
       </c>
@@ -1673,7 +1673,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>49</v>
       </c>
@@ -1699,7 +1699,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>52</v>
       </c>
@@ -1725,7 +1725,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>56</v>
       </c>
@@ -1751,7 +1751,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>59</v>
       </c>
@@ -1777,7 +1777,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>62</v>
       </c>
@@ -1803,7 +1803,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>65</v>
       </c>
@@ -1829,7 +1829,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>68</v>
       </c>
@@ -1849,7 +1849,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>70</v>
       </c>
@@ -1875,7 +1875,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>73</v>
       </c>
@@ -1901,7 +1901,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>77</v>
       </c>
@@ -1927,7 +1927,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>80</v>
       </c>
@@ -1953,7 +1953,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>83</v>
       </c>
@@ -1979,7 +1979,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>86</v>
       </c>
@@ -2005,7 +2005,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>89</v>
       </c>
@@ -2031,7 +2031,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>92</v>
       </c>
@@ -2057,7 +2057,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>95</v>
       </c>
@@ -2083,7 +2083,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>97</v>
       </c>
@@ -2109,7 +2109,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>100</v>
       </c>
@@ -2135,7 +2135,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>103</v>
       </c>
@@ -2161,7 +2161,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>106</v>
       </c>
@@ -2187,7 +2187,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>110</v>
       </c>
@@ -2213,7 +2213,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>112</v>
       </c>
@@ -2239,7 +2239,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>115</v>
       </c>
@@ -2265,7 +2265,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>118</v>
       </c>
@@ -2291,7 +2291,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>121</v>
       </c>
@@ -2317,7 +2317,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>124</v>
       </c>
@@ -2343,7 +2343,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>127</v>
       </c>
@@ -2357,7 +2357,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>129</v>
       </c>
@@ -2383,7 +2383,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>133</v>
       </c>
@@ -2409,7 +2409,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>135</v>
       </c>
@@ -2435,7 +2435,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>138</v>
       </c>
@@ -2461,7 +2461,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>140</v>
       </c>
@@ -2487,7 +2487,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>143</v>
       </c>
@@ -2513,7 +2513,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>146</v>
       </c>
@@ -2539,7 +2539,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>149</v>
       </c>
@@ -2565,7 +2565,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>153</v>
       </c>
@@ -2591,7 +2591,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>156</v>
       </c>
@@ -2617,7 +2617,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>159</v>
       </c>
@@ -2643,7 +2643,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>161</v>
       </c>
@@ -2669,7 +2669,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>165</v>
       </c>
@@ -2695,7 +2695,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>167</v>
       </c>
@@ -2721,7 +2721,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>170</v>
       </c>
@@ -2747,7 +2747,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>218</v>
       </c>
@@ -2773,7 +2773,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>174</v>
       </c>
@@ -2799,7 +2799,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>177</v>
       </c>
@@ -2825,7 +2825,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>179</v>
       </c>
@@ -2851,7 +2851,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>182</v>
       </c>
@@ -2877,7 +2877,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>185</v>
       </c>
@@ -2903,7 +2903,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>188</v>
       </c>
@@ -2929,7 +2929,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>192</v>
       </c>
@@ -2955,7 +2955,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>194</v>
       </c>
@@ -2981,7 +2981,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>197</v>
       </c>
@@ -3007,7 +3007,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>200</v>
       </c>
@@ -3033,7 +3033,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>203</v>
       </c>
@@ -3059,7 +3059,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>206</v>
       </c>
@@ -3085,7 +3085,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>209</v>
       </c>

</xml_diff>